<commit_message>
FEATURE: ya se pueden cargar productos de fomra masiva con un formato de excel y en un segundo paso de sincronización se agregan las fotografías a los productos en tiendanube.
</commit_message>
<xml_diff>
--- a/ProyectoEjecutivo/ContextoDiario-2026-03-15/informeNotebookML-Perfumes_rev01.xlsx
+++ b/ProyectoEjecutivo/ContextoDiario-2026-03-15/informeNotebookML-Perfumes_rev01.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\Proyectos\GeminiTests\AppPerPel\ProyectoEjecutivo\Tiendanube\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\andre\Documents\Proyectos\GeminiTests\AppPerPel\ProyectoEjecutivo\ContextoDiario-2026-03-15\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D03FD19E-F7D8-4ABB-B94E-C6B9D3D5ADE5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B0E8F94-63E2-4A29-9A88-8724063C3884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{968BD831-5A7C-4F25-A2DB-94CC7758444F}"/>
   </bookViews>
@@ -4941,8 +4941,8 @@
     <tableColumn id="9" xr3:uid="{E844D325-0C7A-4FE7-854A-3F658328CAF2}" name="Valor de propiedad 2"/>
     <tableColumn id="10" xr3:uid="{A50AA4F7-2781-4D80-A2FE-065D09AD7E3B}" name="Nombre de propiedad 3"/>
     <tableColumn id="11" xr3:uid="{5F482B42-6924-4A9E-8E54-5C53E2FC572D}" name="Valor de propiedad 3"/>
-    <tableColumn id="12" xr3:uid="{8D5795A9-2020-4436-BE29-66DFAA36F597}" name="Precio" dataDxfId="0"/>
-    <tableColumn id="13" xr3:uid="{9643CFE2-C665-48A7-9C2D-D0EC38408C28}" name="Precio promocional" dataDxfId="2">
+    <tableColumn id="12" xr3:uid="{8D5795A9-2020-4436-BE29-66DFAA36F597}" name="Precio" dataDxfId="2"/>
+    <tableColumn id="13" xr3:uid="{9643CFE2-C665-48A7-9C2D-D0EC38408C28}" name="Precio promocional" dataDxfId="1">
       <calculatedColumnFormula>+Table1[[#This Row],[Precio]]*0.95</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="14" xr3:uid="{C443530D-CF0B-4C90-88E5-A7960CB6BFD1}" name="Peso (kg)"/>
@@ -4963,7 +4963,7 @@
     <tableColumn id="29" xr3:uid="{1943D552-C12B-42A1-B128-42BA890A7BCA}" name="MPN"/>
     <tableColumn id="30" xr3:uid="{14B27409-CAE7-4D1C-A1B7-665224D7527A}" name="Sexo"/>
     <tableColumn id="31" xr3:uid="{1C2AC050-A6ED-4002-B366-828CCC100856}" name="Rango de edad"/>
-    <tableColumn id="32" xr3:uid="{8ECA8A0D-7B54-48C5-B7DC-E7300440527D}" name="Costo" dataDxfId="1">
+    <tableColumn id="32" xr3:uid="{8ECA8A0D-7B54-48C5-B7DC-E7300440527D}" name="Costo" dataDxfId="0">
       <calculatedColumnFormula>+Table1[[#This Row],[Precio]]*0.7</calculatedColumnFormula>
     </tableColumn>
     <tableColumn id="33" xr3:uid="{B1A319F0-10F4-48D2-A861-347C93940FDA}" name="image_url"/>

</xml_diff>